<commit_message>
feat: read-only supplier directory endpoint (GET /api/suppliers)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/document/Feature_Estimation_SCADA_ProjectTracking.xlsx
+++ b/document/Feature_Estimation_SCADA_ProjectTracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milln\CWN Work\Project-Tracking\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F1BF10-0883-47D4-BB67-F85083AA198A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912A24B6-7B41-4DB8-96BE-488D96F14895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="14880" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,9 @@
     <sheet name="Custom vs SaaS" sheetId="3" r:id="rId3"/>
     <sheet name="References" sheetId="4" r:id="rId4"/>
     <sheet name="Chart" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="7" r:id="rId6"/>
-    <sheet name="_chartdata" sheetId="6" state="hidden" r:id="rId7"/>
+    <sheet name="cat_type" sheetId="7" r:id="rId6"/>
+    <sheet name="supplier" sheetId="8" r:id="rId7"/>
+    <sheet name="_chartdata" sheetId="6" state="hidden" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="175">
   <si>
     <t>Feature-Based Estimation — สมมติฐาน (Assumptions)</t>
   </si>
@@ -529,6 +530,33 @@
   </si>
   <si>
     <t>Bar, Ring , Dome, UV</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>sup_name</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>tax_id</t>
+  </si>
+  <si>
+    <t>telephone</t>
+  </si>
+  <si>
+    <t>mobile</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>website</t>
   </si>
 </sst>
 </file>
@@ -795,6 +823,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -804,7 +833,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1505,15 +1533,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
@@ -1953,56 +1981,56 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B23" s="34" t="s">
+      <c r="B23" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
       <c r="F23" s="19">
         <v>1692000</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
       <c r="F24" s="19">
         <v>253800</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B25" s="36" t="s">
+      <c r="B25" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="20">
         <v>1945800</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="21">
         <v>1513400</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B27" s="33" t="s">
+      <c r="B27" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
       <c r="F27" s="22">
         <v>2594400</v>
       </c>
@@ -2032,12 +2060,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
     </row>
     <row r="4" spans="2:5" ht="28.2" x14ac:dyDescent="0.3">
       <c r="B4" s="23" t="s">
@@ -2147,10 +2175,10 @@
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="39" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="39"/>
+      <c r="C5" s="40"/>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
@@ -2193,10 +2221,10 @@
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="C12" s="39"/>
+      <c r="C12" s="40"/>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
@@ -2239,10 +2267,10 @@
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="39" t="s">
         <v>111</v>
       </c>
-      <c r="C19" s="39"/>
+      <c r="C19" s="40"/>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
@@ -2413,7 +2441,7 @@
       <c r="A14" t="s">
         <v>148</v>
       </c>
-      <c r="C14" s="40" t="s">
+      <c r="C14" s="31" t="s">
         <v>162</v>
       </c>
     </row>
@@ -2449,6 +2477,64 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8DB1AB8-BB41-4A8A-AE55-200E0DDD1AD7}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>170</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>